<commit_message>
Excel uyumluluğunu düzelt: CSV, alternatif XLSX ve HTML ekle
XLSX açılmama ihtimaline karşı UTF-8 BOM CSV (noktalı virgül),
xlsxwriter ile ikinci XLSX ve tarayıcıda açılan HTML liste eklendi.

Co-authored-by: Smdaer <Smdaer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/O_bir_defineci_videolar.xlsx
+++ b/O_bir_defineci_videolar.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="O bir defineci" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Videolar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ozet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'O bir defineci'!$A$1:$G$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Videolar'!$A$1:$G$294</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
@@ -483,32 +483,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Sanatçı / Ses Sahibi</t>
+          <t>Sanatci / Ses Sahibi</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Parça / Ses Adı</t>
+          <t>Parca / Ses Adi</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Açıklama / Hashtagler</t>
+          <t>Aciklama / Hashtagler</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Görüntülenme</t>
+          <t>Goruntulenme</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Görüntülenme (Sayı)</t>
+          <t>Goruntulenme (Sayi)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Oluşturan</t>
+          <t>Olusturan</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10014,7 +10014,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Özet</t>
+          <t>Ozet</t>
         </is>
       </c>
     </row>
@@ -10031,110 +10031,123 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Görüntülenmesi olan</t>
+          <t>Toplam goruntulenme (yaklasik)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Toplam görüntülenme (yaklaşık)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
         <v>2944624</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>En cok goruntulenen 20</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>En çok görüntülenen 20 video</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Sanatci</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Parca</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Goruntulenme</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Sayi</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Sanatçı</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Parça</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Görüntülenme</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Sayı</t>
-        </is>
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Levent Aktaş</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>orijinal ses</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>75.3K</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>75300</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Levent Aktaş</t>
+          <t>kurdarchive</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>orijinal ses</t>
+          <t>kurdarchive - orijinal ses</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>75.3K</t>
+          <t>74.8K</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>75300</v>
+        <v>74800</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>kurdarchive</t>
+          <t>Hewidar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kurdarchive - orijinal ses</t>
+          <t>orijinal ses</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>74.8K</t>
+          <t>56.4K</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>74800</v>
+        <v>56400</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hewidar</t>
+          <t>Denge Kurdi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -10144,20 +10157,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>56.4K</t>
+          <t>50K</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>56400</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Denge Kurdi</t>
+          <t>Rojda şenses</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -10167,20 +10180,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>50K</t>
+          <t>48K</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>50000</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rojda şenses</t>
+          <t>illegalask_62</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -10190,20 +10203,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48K</t>
+          <t>46.1K</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>48000</v>
+        <v>46100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>illegalask_62</t>
+          <t>🎶MUHAMMET ARAS🎶FAN</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -10213,20 +10226,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>46.1K</t>
+          <t>44.5K</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46100</v>
+        <v>44500</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>🎶MUHAMMET ARAS🎶FAN</t>
+          <t>Meral Alkan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -10236,20 +10249,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>44.5K</t>
+          <t>44.1K</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>44500</v>
+        <v>44100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meral Alkan</t>
+          <t>Ɓeysu Ɓaşkan✌️📿</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -10259,20 +10272,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>44.1K</t>
+          <t>43K</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>44100</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ɓeysu Ɓaşkan✌️📿</t>
+          <t>user49655852229</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -10282,58 +10295,58 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>43K</t>
+          <t>39.2K</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>43000</v>
+        <v>39200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>user49655852229</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>orijinal ses</t>
-        </is>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>39.2K</t>
+          <t>38.1K</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>39200</v>
+        <v>38100</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>user98728770565</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>الصوت الأصلي</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>38.1K</t>
+          <t>37.4K</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>38100</v>
+        <v>37400</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>user98728770565</t>
+          <t>ابو رودي</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -10343,112 +10356,112 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>37.4K</t>
+          <t>35.4K</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>37400</v>
+        <v>35400</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ابو رودي</t>
+          <t>Alevi✌️im</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>الصوت الأصلي</t>
+          <t>Originalton</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>35.4K</t>
+          <t>35.2K</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>35400</v>
+        <v>35200</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alevi✌️im</t>
+          <t>merwan968</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Originalton</t>
+          <t>orijinal ses</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>35.2K</t>
+          <t>34.2K</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>35200</v>
+        <v>34200</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>merwan968</t>
+          <t>Efrîna min</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>orijinal ses</t>
+          <t>الصوت الأصلي</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>34.2K</t>
+          <t>33.7K</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>34200</v>
+        <v>33700</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Efrîna min</t>
+          <t>HEWİ✌🏿🖤🥀</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>الصوت الأصلي</t>
+          <t>orijinal ses</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>33.7K</t>
+          <t>33.6K</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>33700</v>
+        <v>33600</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HEWİ✌🏿🖤🥀</t>
+          <t>O bir defineci</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -10458,20 +10471,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>33.6K</t>
+          <t>32.6K</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>33600</v>
+        <v>32600</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>O bir defineci</t>
+          <t>delildilanarofficial</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -10481,20 +10494,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>32.6K</t>
+          <t>32K</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>32600</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>delildilanarofficial</t>
+          <t>O bir defineci</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -10504,33 +10517,10 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>32K</t>
+          <t>30.7K</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>O bir defineci</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>orijinal ses</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>30.7K</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
         <v>30700</v>
       </c>
     </row>

</xml_diff>